<commit_message>
docs: update Phase3  280126
</commit_message>
<xml_diff>
--- a/results/phase1/FT_26/config_FT_cr_240126.xlsx
+++ b/results/phase1/FT_26/config_FT_cr_240126.xlsx
@@ -481,7 +481,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:B12"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.19140625" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.21875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15.8" customWidth="1" style="6" min="1" max="1"/>
   </cols>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" ht="13.5" customHeight="1" s="7">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="13.5" customHeight="1" s="7">
@@ -637,7 +637,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:I429"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.5625" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.578125" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12.71" customWidth="1" style="6" min="2" max="2"/>
     <col width="13.26" customWidth="1" style="6" min="3" max="3"/>
@@ -3854,8 +3854,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q10"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:Q11"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.70703125" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="7">
       <c r="A1" s="6" t="inlineStr">
@@ -4343,7 +4343,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="15" customHeight="1" s="7">
       <c r="A9" s="6" t="n">
         <v>0</v>
       </c>
@@ -4356,13 +4356,13 @@
         <v>8</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0.01034453976899385</v>
+        <v>0.0103445397689939</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>0.998</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.06206387281417847</v>
+        <v>0.0620638728141785</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>0.988</v>
@@ -4379,13 +4379,13 @@
       <c r="K9" s="6" t="n">
         <v>0.986</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="L9" s="10" t="n">
         <v>46047.51592592592</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="M9" s="10" t="n">
         <v>46047.54689814815</v>
       </c>
-      <c r="N9" s="13" t="n">
+      <c r="N9" s="11" t="n">
         <v>0.03097222222222222</v>
       </c>
       <c r="O9" s="6" t="n">
@@ -4400,58 +4400,115 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="n">
+    <row r="10" ht="15" customHeight="1" s="7">
+      <c r="A10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>DenseNet201</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="D10" t="n">
-        <v>0.01489091850817204</v>
-      </c>
-      <c r="E10" t="n">
+      <c r="D10" s="6" t="n">
+        <v>0.014890918508172</v>
+      </c>
+      <c r="E10" s="6" t="n">
         <v>0.995</v>
       </c>
-      <c r="F10" t="n">
-        <v>0.1431334018707275</v>
-      </c>
-      <c r="G10" t="n">
+      <c r="F10" s="6" t="n">
+        <v>0.143133401870728</v>
+      </c>
+      <c r="G10" s="6" t="n">
         <v>0.973</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="6" t="n">
         <v>0.974</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" s="6" t="n">
         <v>0.973</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J10" s="6" t="n">
         <v>0.972</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" s="6" t="n">
         <v>0.969</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="L10" s="10" t="n">
         <v>46047.5471412037</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="M10" s="10" t="n">
         <v>46047.58346064815</v>
       </c>
-      <c r="N10" s="13" t="n">
+      <c r="N10" s="11" t="n">
         <v>0.03631944444444445</v>
       </c>
-      <c r="O10" t="n">
+      <c r="O10" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P10" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="Q10" s="6" t="inlineStr">
+        <is>
+          <t>FT_DFT_K10_xlsx.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>0</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DenseNet201</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.0227500181645155</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.1042143329977989</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.978</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.978</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.978</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>46049.53267361111</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>46049.55561342592</v>
+      </c>
+      <c r="N11" s="13" t="n">
+        <v>0.02293981481481482</v>
+      </c>
+      <c r="O11" t="n">
+        <v>9</v>
+      </c>
+      <c r="P11" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>FT_DFT_K10_xlsx.py</t>
         </is>

</xml_diff>